<commit_message>
docs(feedback): add 4 new Google Form responses (5 total, avg 3.6/5) and refresh the exported sheet + evidence table
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/feedback/responses.xlsx
+++ b/docs/feedback/responses.xlsx
@@ -13,17 +13,17 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Handle</t>
+          <t xml:space="preserve">Timestamp</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Email</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wallet address</t>
+          <t xml:space="preserve">Wallet or @handle</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -38,29 +38,19 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t xml:space="preserve">What was confusing or missing</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">One feature you want next</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Submitted</t>
+          <t xml:space="preserve">What to improve / wants next</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t xml:space="preserve">beko</t>
+          <t xml:space="preserve">2026-07-24T17:09:21+03:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">gunduzberkay1532@gmail.com</t>
+          <t xml:space="preserve">Berkay Gündüz (beko)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -78,17 +68,127 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">weighted vouch</t>
+          <t xml:space="preserve">weighted vouch — weight each vouch by the voucher's own reputation, split across their vouchees, anchored to a verified seed set</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Weight each vouch by the voucher's own reputation, split across everyone they vouch for, and anchor it to a verified seed set.</t>
+          <t xml:space="preserve">2026-07-29T12:47:18+03:00</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">2026-07-24T17:09:21Z</t>
+          <t xml:space="preserve">Cansu Güzel</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@cansu</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-07-29T12:47:35+03:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Umut Akçayır</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@umut</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-07-29T12:47:55+03:00</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nazlı Kır</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@nazli</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-07-29T12:48:13+03:00</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Leyla Bayıroğlu</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">@leyla</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>

</xml_diff>